<commit_message>
Résolution des conflits 703bcb9d72967e7098d27b7cb4edab4347acb933
</commit_message>
<xml_diff>
--- a/HTR-IGDoc/ig/StructureDefinition-fr-Organization-document.xlsx
+++ b/HTR-IGDoc/ig/StructureDefinition-fr-Organization-document.xlsx
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-18T10:06:11+00:00</t>
+    <t>2025-02-18T11:00:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2598,7 +2598,7 @@
         <v>77</v>
       </c>
       <c r="G13" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H13" t="s" s="2">
         <v>76</v>

</xml_diff>